<commit_message>
add update for fake file list
</commit_message>
<xml_diff>
--- a/doc/OneNode数据格式.xlsx
+++ b/doc/OneNode数据格式.xlsx
@@ -4,12 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375" activeTab="2"/>
+    <workbookView windowHeight="17895" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Message" sheetId="1" r:id="rId1"/>
     <sheet name="IOData" sheetId="2" r:id="rId2"/>
-    <sheet name="ApplicationState" sheetId="4" r:id="rId3"/>
+    <sheet name="API" sheetId="5" r:id="rId3"/>
+    <sheet name="builtin" sheetId="6" r:id="rId4"/>
+    <sheet name="ApplicationState" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="112">
   <si>
     <t>字段</t>
   </si>
@@ -37,6 +39,9 @@
     <t>取值格式</t>
   </si>
   <si>
+    <t>数据类型</t>
+  </si>
+  <si>
     <t>定义</t>
   </si>
   <si>
@@ -50,6 +55,9 @@
   </si>
   <si>
     <t>prompt</t>
+  </si>
+  <si>
+    <t>字符串</t>
   </si>
   <si>
     <t>做什么事，做事过程中需要用户知道的，执行中间状态</t>
@@ -168,7 +176,17 @@
     <t>file</t>
   </si>
   <si>
+    <t>文件名字符串</t>
+  </si>
+  <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>data返回文件key，</t>
     </r>
     <r>
@@ -193,6 +211,12 @@
     </r>
   </si>
   <si>
+    <t>files</t>
+  </si>
+  <si>
+    <t>文件名字符串列表</t>
+  </si>
+  <si>
     <t>chart</t>
   </si>
   <si>
@@ -305,6 +329,148 @@
   </si>
   <si>
     <t>[{"status": "error", "type": "markdown", "data": "{其它项目_进度概况} - 数据未就绪"}]</t>
+  </si>
+  <si>
+    <t>导入文件列表</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>https://www.seek-time.com:43031/agents/api/v1/application/run</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>{
+  "option":  {
+     "page": 1，
+     "page_length": 12,
+     "filter": {
+           "fetch_state": null/success/failed,
+           "import_state": null/success/failed
+      }
+  },
+  "app_name": "公估报告智数问答",
+  "agent_name": "问题解析",
+  "new_ctx": false
+}</t>
+  </si>
+  <si>
+    <t>Response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+{
+"channel": "response", 
+"command": "append", 
+"app_name":"智数问答"
+"agent_name":"读取同步文件名列表"
+"role": "agent:\u8bfb\u53d6\u6587\u4ef6\u5217\u8868", 
+"data": 
+     {
+            "app_id": "680icft5uw3o", 
+            "agent_id": "0dtia1srsnv4", 
+            "type": "files", 
+            "content": [
+                 "xxxxx",
+                  "yyyy",
+                 "zzzz"
+            ]
+    }, 
+"thread": ""
+}</t>
+  </si>
+  <si>
+    <t>文件列表可能分几次给出，在退去调用前，前端需要收集content中的文件列表
+前端只需要捕捉预定的agent_name名的消息，忽略其它的消息</t>
+  </si>
+  <si>
+    <t>bu</t>
+  </si>
+  <si>
+    <t>当前函数名</t>
+  </si>
+  <si>
+    <t>新函数名</t>
+  </si>
+  <si>
+    <t>参数</t>
+  </si>
+  <si>
+    <t>功能定义</t>
+  </si>
+  <si>
+    <t>get_nodes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ctx: 当前上下文
+name: 数据节点名字
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>label: 标签名</t>
+    </r>
+  </si>
+  <si>
+    <t>取当前上下文中指定名字的data节点下的子节点列表</t>
+  </si>
+  <si>
+    <t>save_io_data</t>
+  </si>
+  <si>
+    <t>save_data</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ctx: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>当前上下文 (如果为空，刚放置到全局)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+name: 数据节点名字
+data: 不要限定为markdown</t>
+    </r>
+  </si>
+  <si>
+    <t>clear_output()不能调，是bug</t>
+  </si>
+  <si>
+    <t>anext_agent</t>
+  </si>
+  <si>
+    <t>aprint_message</t>
+  </si>
+  <si>
+    <t>aprint_response</t>
+  </si>
+  <si>
+    <t>end_flow</t>
   </si>
 </sst>
 </file>
@@ -312,10 +478,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -326,16 +492,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -691,7 +857,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -858,17 +1024,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -971,19 +1126,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -992,7 +1147,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1004,34 +1159,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1116,12 +1271,27 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
@@ -1135,9 +1305,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1159,13 +1326,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1174,34 +1338,19 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1216,44 +1365,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1267,9 +1398,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1279,37 +1407,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1318,10 +1440,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1330,12 +1449,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1345,32 +1458,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1900,339 +2001,407 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:G27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="24" customHeight="1" outlineLevelCol="6"/>
+  <dimension ref="B1:H28"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="24" customHeight="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="9" style="24"/>
-    <col min="2" max="2" width="14" style="25" customWidth="1"/>
-    <col min="3" max="3" width="15.5" style="25" customWidth="1"/>
-    <col min="4" max="4" width="18.5" style="25" customWidth="1"/>
-    <col min="5" max="5" width="73.75" style="25" customWidth="1"/>
-    <col min="6" max="6" width="43.625" style="25" customWidth="1"/>
-    <col min="7" max="7" width="33.25" style="25" customWidth="1"/>
-    <col min="8" max="8" width="41.5" style="25" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="24"/>
+    <col min="1" max="1" width="9" style="23"/>
+    <col min="2" max="2" width="14" style="23" customWidth="1"/>
+    <col min="3" max="3" width="15.5" style="23" customWidth="1"/>
+    <col min="4" max="5" width="18.5" style="23" customWidth="1"/>
+    <col min="6" max="6" width="73.75" style="23" customWidth="1"/>
+    <col min="7" max="7" width="43.625" style="23" customWidth="1"/>
+    <col min="8" max="8" width="33.25" style="23" customWidth="1"/>
+    <col min="9" max="9" width="41.5" style="23" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="2:7">
-      <c r="B1" s="26" t="s">
+    <row r="1" customHeight="1" spans="2:8">
+      <c r="B1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28"/>
+      <c r="D1" s="26"/>
       <c r="E1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="24" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" customHeight="1" spans="2:7">
-      <c r="B2" s="29" t="s">
+      <c r="H1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="30" t="s">
+    </row>
+    <row r="2" customHeight="1" spans="2:8">
+      <c r="B2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="32" t="s">
+      <c r="C2" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="33"/>
-      <c r="G2" s="34"/>
-    </row>
-    <row r="3" customHeight="1" spans="2:7">
-      <c r="B3" s="35"/>
-      <c r="C3" s="36" t="s">
+      <c r="D2" s="29"/>
+      <c r="E2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="38" t="s">
+      <c r="F2" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="39"/>
-      <c r="G3" s="40"/>
-    </row>
-    <row r="4" customHeight="1" spans="2:7">
-      <c r="B4" s="35"/>
-      <c r="C4" s="41" t="s">
+      <c r="G2" s="30"/>
+      <c r="H2" s="31"/>
+    </row>
+    <row r="3" customHeight="1" spans="2:8">
+      <c r="B3" s="32"/>
+      <c r="C3" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="38" t="s">
+      <c r="D3" s="34"/>
+      <c r="E3" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="39"/>
-      <c r="G4" s="40"/>
-    </row>
-    <row r="5" customHeight="1" spans="2:7">
-      <c r="B5" s="35"/>
-      <c r="C5" s="43" t="s">
+      <c r="H3" s="36"/>
+    </row>
+    <row r="4" customHeight="1" spans="2:8">
+      <c r="B4" s="32"/>
+      <c r="C4" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="38" t="s">
+      <c r="D4" s="34"/>
+      <c r="E4" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="40"/>
-    </row>
-    <row r="6" customHeight="1" spans="2:7">
-      <c r="B6" s="46"/>
-      <c r="C6" s="47" t="s">
+      <c r="H4" s="36"/>
+    </row>
+    <row r="5" customHeight="1" spans="2:8">
+      <c r="B5" s="32"/>
+      <c r="C5" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="48"/>
-      <c r="E6" s="49" t="s">
+      <c r="D5" s="37"/>
+      <c r="E5" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="50"/>
-      <c r="G6" s="51"/>
-    </row>
-    <row r="7" customHeight="1" spans="2:7">
-      <c r="B7" s="29" t="s">
+      <c r="H5" s="36"/>
+    </row>
+    <row r="6" customHeight="1" spans="2:8">
+      <c r="B6" s="38"/>
+      <c r="C6" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="D6" s="40"/>
+      <c r="E6" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="53"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="34"/>
-    </row>
-    <row r="8" customHeight="1" spans="2:7">
-      <c r="B8" s="35"/>
-      <c r="C8" s="54" t="s">
+      <c r="G6" s="41"/>
+      <c r="H6" s="42"/>
+    </row>
+    <row r="7" customHeight="1" spans="2:8">
+      <c r="B7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="55"/>
-      <c r="E8" s="56"/>
-      <c r="G8" s="56"/>
-    </row>
-    <row r="9" customHeight="1" spans="2:7">
-      <c r="B9" s="35"/>
-      <c r="C9" s="54" t="s">
+      <c r="C7" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="55"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="58"/>
-      <c r="G9" s="56"/>
-    </row>
-    <row r="10" customHeight="1" spans="2:7">
-      <c r="B10" s="46"/>
-      <c r="C10" s="59" t="s">
+      <c r="D7" s="44"/>
+      <c r="E7" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31"/>
+    </row>
+    <row r="8" customHeight="1" spans="2:8">
+      <c r="B8" s="32"/>
+      <c r="C8" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="60"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="51"/>
-    </row>
-    <row r="11" customHeight="1" spans="2:7">
-      <c r="B11" s="29" t="s">
+      <c r="D8" s="46"/>
+      <c r="E8" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="36"/>
+      <c r="H8" s="36"/>
+    </row>
+    <row r="9" customHeight="1" spans="2:8">
+      <c r="B9" s="32"/>
+      <c r="C9" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="D9" s="46"/>
+      <c r="E9" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="47"/>
+      <c r="G9" s="47"/>
+      <c r="H9" s="36"/>
+    </row>
+    <row r="10" customHeight="1" spans="2:8">
+      <c r="B10" s="38"/>
+      <c r="C10" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="62"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34" t="s">
+      <c r="D10" s="49"/>
+      <c r="E10" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="42"/>
+    </row>
+    <row r="11" customHeight="1" spans="2:8">
+      <c r="B11" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="63" t="s">
+      <c r="C11" s="50" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" customHeight="1" spans="2:7">
-      <c r="B12" s="35"/>
-      <c r="C12" s="54" t="s">
+      <c r="D11" s="51"/>
+      <c r="E11" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="64"/>
-      <c r="E12" s="56"/>
-      <c r="F12" s="56" t="s">
+      <c r="H11" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="65"/>
-    </row>
-    <row r="13" customHeight="1" spans="2:7">
-      <c r="B13" s="35"/>
-      <c r="C13" s="54" t="s">
+    </row>
+    <row r="12" customHeight="1" spans="2:8">
+      <c r="B12" s="32"/>
+      <c r="C12" s="45" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="64"/>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56" t="s">
+      <c r="D12" s="53"/>
+      <c r="E12" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="65"/>
-    </row>
-    <row r="14" customHeight="1" spans="2:7">
-      <c r="B14" s="35"/>
-      <c r="C14" s="54" t="s">
+      <c r="H12" s="54"/>
+    </row>
+    <row r="13" customHeight="1" spans="2:8">
+      <c r="B13" s="32"/>
+      <c r="C13" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="64"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56" t="s">
+      <c r="D13" s="53"/>
+      <c r="E13" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="65"/>
-    </row>
-    <row r="15" customHeight="1" spans="2:7">
-      <c r="B15" s="35"/>
-      <c r="C15" s="54" t="s">
+      <c r="H13" s="54"/>
+    </row>
+    <row r="14" customHeight="1" spans="2:8">
+      <c r="B14" s="32"/>
+      <c r="C14" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="64"/>
-      <c r="E15" s="56" t="s">
+      <c r="D14" s="53"/>
+      <c r="E14" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="56" t="s">
+      <c r="H14" s="54"/>
+    </row>
+    <row r="15" customHeight="1" spans="2:8">
+      <c r="B15" s="32"/>
+      <c r="C15" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="65"/>
-    </row>
-    <row r="16" customHeight="1" spans="2:7">
-      <c r="B16" s="66" t="s">
+      <c r="D15" s="53"/>
+      <c r="E15" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="67" t="s">
+      <c r="G15" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="68" t="s">
+      <c r="H15" s="54"/>
+    </row>
+    <row r="16" customHeight="1" spans="2:8">
+      <c r="B16" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="66"/>
-      <c r="F16" s="69" t="s">
+      <c r="C16" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="70" t="s">
+      <c r="D16" s="56" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" customHeight="1" spans="2:7">
-      <c r="B17" s="35"/>
-      <c r="C17" s="71"/>
-      <c r="D17" s="72" t="s">
+      <c r="E16" s="56"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="73" t="s">
+      <c r="H16" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="74"/>
-      <c r="G17" s="75"/>
-    </row>
-    <row r="18" customHeight="1" spans="2:7">
-      <c r="B18" s="35"/>
-      <c r="C18" s="71"/>
-      <c r="D18" s="72" t="s">
+    </row>
+    <row r="17" customHeight="1" spans="2:8">
+      <c r="B17" s="32"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="73"/>
-      <c r="F18" s="74"/>
-      <c r="G18" s="75"/>
-    </row>
-    <row r="19" customHeight="1" spans="2:7">
-      <c r="B19" s="35"/>
-      <c r="C19" s="71"/>
-      <c r="D19" s="76" t="s">
+      <c r="E17" s="56"/>
+      <c r="F17" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="73"/>
-      <c r="F19" s="74"/>
-      <c r="G19" s="75"/>
-    </row>
-    <row r="20" customHeight="1" spans="2:7">
-      <c r="B20" s="35"/>
-      <c r="C20" s="71"/>
-      <c r="D20" s="76" t="s">
+      <c r="G17" s="60"/>
+      <c r="H17" s="61"/>
+    </row>
+    <row r="18" customHeight="1" spans="2:8">
+      <c r="B18" s="32"/>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="77" t="s">
+      <c r="E18" s="56"/>
+      <c r="F18" s="59"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="61"/>
+    </row>
+    <row r="19" customHeight="1" spans="2:8">
+      <c r="B19" s="32"/>
+      <c r="C19" s="56"/>
+      <c r="D19" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="F20" s="74"/>
-      <c r="G20" s="75"/>
-    </row>
-    <row r="21" customHeight="1" spans="2:7">
-      <c r="B21" s="35"/>
-      <c r="C21" s="71"/>
-      <c r="D21" s="44" t="s">
+      <c r="E19" s="62"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="60"/>
+      <c r="H19" s="61"/>
+    </row>
+    <row r="20" customHeight="1" spans="2:8">
+      <c r="B20" s="32"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="74" t="s">
+      <c r="E20" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="F21" s="74"/>
-      <c r="G21" s="75"/>
-    </row>
-    <row r="22" customHeight="1" spans="2:7">
-      <c r="B22" s="35"/>
-      <c r="C22" s="71"/>
-      <c r="D22" s="78" t="s">
+      <c r="F20" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="74"/>
-      <c r="F22" s="74"/>
-      <c r="G22" s="75"/>
-    </row>
-    <row r="23" customHeight="1" spans="2:7">
-      <c r="B23" s="35"/>
-      <c r="C23" s="71"/>
-      <c r="D23" s="78" t="s">
+      <c r="G20" s="60"/>
+      <c r="H20" s="61"/>
+    </row>
+    <row r="21" customHeight="1" spans="2:8">
+      <c r="B21" s="32"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="E23" s="74"/>
-      <c r="F23" s="74"/>
-      <c r="G23" s="75"/>
-    </row>
-    <row r="24" customHeight="1" spans="2:7">
-      <c r="B24" s="35"/>
-      <c r="C24" s="79"/>
-      <c r="D24" s="78" t="s">
+      <c r="E21" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="75"/>
-    </row>
-    <row r="25" customHeight="1" spans="2:7">
-      <c r="B25" s="35"/>
-      <c r="C25" s="80" t="s">
+      <c r="F21" s="63"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="61"/>
+    </row>
+    <row r="22" customHeight="1" spans="2:8">
+      <c r="B22" s="32"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="D25" s="81" t="s">
+      <c r="E22" s="62"/>
+      <c r="F22" s="60" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="74"/>
-      <c r="F25" s="74"/>
-      <c r="G25" s="82"/>
-    </row>
-    <row r="26" customHeight="1" spans="2:7">
-      <c r="B26" s="83" t="s">
+      <c r="G22" s="60"/>
+      <c r="H22" s="61"/>
+    </row>
+    <row r="23" customHeight="1" spans="2:8">
+      <c r="B23" s="32"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="47" t="s">
+      <c r="E23" s="64"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="61"/>
+    </row>
+    <row r="24" customHeight="1" spans="2:8">
+      <c r="B24" s="32"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="64" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="84"/>
-      <c r="E26" s="80"/>
-      <c r="F26" s="80" t="s">
+      <c r="E24" s="64"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="60"/>
+      <c r="H24" s="61"/>
+    </row>
+    <row r="25" customHeight="1" spans="2:8">
+      <c r="B25" s="32"/>
+      <c r="C25" s="56"/>
+      <c r="D25" s="64" t="s">
         <v>54</v>
       </c>
-      <c r="G26" s="51"/>
-    </row>
-    <row r="27" customHeight="1" spans="2:7">
-      <c r="B27" s="85"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="60"/>
+      <c r="H25" s="61"/>
+    </row>
+    <row r="26" customHeight="1" spans="2:8">
+      <c r="B26" s="32"/>
+      <c r="C26" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="56" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="56"/>
+      <c r="F26" s="60"/>
+      <c r="G26" s="60"/>
+      <c r="H26" s="66"/>
+    </row>
+    <row r="27" customHeight="1" spans="2:8">
+      <c r="B27" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="D27" s="56"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65" t="s">
+        <v>59</v>
+      </c>
+      <c r="H27" s="42"/>
+    </row>
+    <row r="28" customHeight="1" spans="2:8">
+      <c r="B28" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -2251,16 +2420,16 @@
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
     <mergeCell ref="B2:B6"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="B11:B15"/>
-    <mergeCell ref="B16:B25"/>
-    <mergeCell ref="C16:C24"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F16:F25"/>
-    <mergeCell ref="G11:G15"/>
-    <mergeCell ref="G16:G25"/>
+    <mergeCell ref="B16:B26"/>
+    <mergeCell ref="C16:C25"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G16:G26"/>
+    <mergeCell ref="H11:H15"/>
+    <mergeCell ref="H16:H26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2273,440 +2442,440 @@
   <dimension ref="B1:X28"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="37" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="9" style="2"/>
-    <col min="2" max="2" width="18.125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="19.875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="48.25" style="2" customWidth="1"/>
-    <col min="5" max="5" width="34.75" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="2"/>
+    <col min="1" max="1" width="9" style="7"/>
+    <col min="2" max="2" width="18.125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="19.875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="48.25" style="7" customWidth="1"/>
+    <col min="5" max="5" width="34.75" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="7"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="2:8">
-      <c r="B1" s="2" t="s">
-        <v>55</v>
+      <c r="B1" s="7" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="2:8">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" customHeight="1" spans="2:8">
+      <c r="B3" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+    </row>
+    <row r="4" customHeight="1" spans="2:8">
+      <c r="B4" s="12"/>
+      <c r="C4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" customHeight="1" spans="2:8">
+      <c r="B5" s="12"/>
+      <c r="C5" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" customHeight="1" spans="2:8">
+      <c r="B6" s="13"/>
+      <c r="C6" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" customHeight="1" spans="2:8">
+      <c r="B7" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" customHeight="1" spans="2:8">
+      <c r="B8" s="12"/>
+      <c r="C8" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="13"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" customHeight="1" spans="2:8">
+      <c r="B9" s="12"/>
+      <c r="C9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" customHeight="1" spans="2:8">
+      <c r="B10" s="12"/>
+      <c r="C10" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" customHeight="1" spans="2:8">
+      <c r="B11" s="12"/>
+      <c r="C11" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" customHeight="1" spans="2:8">
+      <c r="B12" s="13"/>
+      <c r="C12" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" customHeight="1" spans="2:8">
+      <c r="B13" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="2:8">
-      <c r="B3" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-    </row>
-    <row r="4" customHeight="1" spans="2:8">
-      <c r="B4" s="8"/>
-      <c r="C4" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" customHeight="1" spans="2:8">
-      <c r="B5" s="8"/>
-      <c r="C5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" customHeight="1" spans="2:8">
-      <c r="B6" s="9"/>
-      <c r="C6" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" customHeight="1" spans="2:8">
-      <c r="B7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" customHeight="1" spans="2:8">
-      <c r="B8" s="8"/>
-      <c r="C8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" customHeight="1" spans="2:8">
-      <c r="B9" s="8"/>
-      <c r="C9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" customHeight="1" spans="2:8">
-      <c r="B10" s="8"/>
-      <c r="C10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" customHeight="1" spans="2:8">
-      <c r="B11" s="8"/>
-      <c r="C11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" customHeight="1" spans="2:8">
-      <c r="B12" s="9"/>
-      <c r="C12" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" customHeight="1" spans="2:8">
-      <c r="B13" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" customHeight="1" spans="2:8">
-      <c r="B14" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="13"/>
+      <c r="B14" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="E14" s="17"/>
     </row>
     <row r="16" customHeight="1" spans="2:8">
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" customHeight="1" spans="2:24">
+      <c r="B17" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="19"/>
+      <c r="S17" s="19"/>
+      <c r="T17" s="19"/>
+      <c r="U17" s="19"/>
+      <c r="V17" s="19"/>
+      <c r="W17" s="19"/>
+      <c r="X17" s="19"/>
+    </row>
+    <row r="18" customHeight="1" spans="2:24">
+      <c r="B18" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="20"/>
+      <c r="M18" s="20"/>
+      <c r="N18" s="20"/>
+      <c r="O18" s="20"/>
+      <c r="P18" s="20"/>
+      <c r="Q18" s="20"/>
+      <c r="R18" s="20"/>
+      <c r="S18" s="20"/>
+      <c r="T18" s="20"/>
+      <c r="U18" s="20"/>
+      <c r="V18" s="20"/>
+      <c r="W18" s="20"/>
+      <c r="X18" s="21"/>
+    </row>
+    <row r="19" customHeight="1" spans="2:24">
+      <c r="B19" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="19"/>
+      <c r="S19" s="19"/>
+      <c r="T19" s="19"/>
+      <c r="U19" s="19"/>
+      <c r="V19" s="19"/>
+      <c r="W19" s="19"/>
+      <c r="X19" s="19"/>
+    </row>
+    <row r="20" customHeight="1" spans="2:24">
+      <c r="B20" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="S20" s="17"/>
+      <c r="T20" s="17"/>
+      <c r="U20" s="17"/>
+      <c r="V20" s="17"/>
+      <c r="W20" s="17"/>
+      <c r="X20" s="17"/>
+    </row>
+    <row r="21" customHeight="1" spans="2:24">
+      <c r="B21" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="17"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="17"/>
+      <c r="S21" s="17"/>
+      <c r="T21" s="17"/>
+      <c r="U21" s="17"/>
+      <c r="V21" s="17"/>
+      <c r="W21" s="17"/>
+      <c r="X21" s="17"/>
+    </row>
+    <row r="22" customHeight="1" spans="2:24">
+      <c r="B22" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="17" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="17" customHeight="1" spans="2:24">
-      <c r="B17" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="16"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="16"/>
-      <c r="Q17" s="16"/>
-      <c r="R17" s="16"/>
-      <c r="S17" s="16"/>
-      <c r="T17" s="16"/>
-      <c r="U17" s="16"/>
-      <c r="V17" s="16"/>
-      <c r="W17" s="16"/>
-      <c r="X17" s="16"/>
-    </row>
-    <row r="18" customHeight="1" spans="2:24">
-      <c r="B18" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="17"/>
-      <c r="U18" s="17"/>
-      <c r="V18" s="17"/>
-      <c r="W18" s="17"/>
-      <c r="X18" s="18"/>
-    </row>
-    <row r="19" customHeight="1" spans="2:24">
-      <c r="B19" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="20"/>
-      <c r="P19" s="20"/>
-      <c r="Q19" s="20"/>
-      <c r="R19" s="20"/>
-      <c r="S19" s="20"/>
-      <c r="T19" s="20"/>
-      <c r="U19" s="20"/>
-      <c r="V19" s="20"/>
-      <c r="W19" s="20"/>
-      <c r="X19" s="20"/>
-    </row>
-    <row r="20" customHeight="1" spans="2:24">
-      <c r="B20" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="21"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="21"/>
-      <c r="P20" s="21"/>
-      <c r="Q20" s="21"/>
-      <c r="R20" s="21"/>
-      <c r="S20" s="21"/>
-      <c r="T20" s="21"/>
-      <c r="U20" s="21"/>
-      <c r="V20" s="21"/>
-      <c r="W20" s="21"/>
-      <c r="X20" s="21"/>
-    </row>
-    <row r="21" customHeight="1" spans="2:24">
-      <c r="B21" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="S21" s="21"/>
-      <c r="T21" s="21"/>
-      <c r="U21" s="21"/>
-      <c r="V21" s="21"/>
-      <c r="W21" s="21"/>
-      <c r="X21" s="21"/>
-    </row>
-    <row r="22" customHeight="1" spans="2:24">
-      <c r="B22" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
-      <c r="O22" s="21"/>
-      <c r="P22" s="21"/>
-      <c r="Q22" s="21"/>
-      <c r="R22" s="21"/>
-      <c r="S22" s="21"/>
-      <c r="T22" s="21"/>
-      <c r="U22" s="21"/>
-      <c r="V22" s="21"/>
-      <c r="W22" s="21"/>
-      <c r="X22" s="21"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="17"/>
+      <c r="M22" s="17"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="17"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="17"/>
+      <c r="S22" s="17"/>
+      <c r="T22" s="17"/>
+      <c r="U22" s="17"/>
+      <c r="V22" s="17"/>
+      <c r="W22" s="17"/>
+      <c r="X22" s="17"/>
     </row>
     <row r="23" customHeight="1" spans="2:24">
-      <c r="B23" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="21"/>
-      <c r="O23" s="21"/>
-      <c r="P23" s="21"/>
-      <c r="Q23" s="21"/>
-      <c r="R23" s="21"/>
-      <c r="S23" s="21"/>
-      <c r="T23" s="21"/>
-      <c r="U23" s="21"/>
-      <c r="V23" s="21"/>
-      <c r="W23" s="21"/>
-      <c r="X23" s="21"/>
+      <c r="B23" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+      <c r="Q23" s="17"/>
+      <c r="R23" s="17"/>
+      <c r="S23" s="17"/>
+      <c r="T23" s="17"/>
+      <c r="U23" s="17"/>
+      <c r="V23" s="17"/>
+      <c r="W23" s="17"/>
+      <c r="X23" s="17"/>
     </row>
     <row r="24" customHeight="1" spans="2:24">
-      <c r="B24" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="21"/>
-      <c r="O24" s="21"/>
-      <c r="P24" s="21"/>
-      <c r="Q24" s="21"/>
-      <c r="R24" s="21"/>
-      <c r="S24" s="21"/>
-      <c r="T24" s="21"/>
-      <c r="U24" s="21"/>
-      <c r="V24" s="21"/>
-      <c r="W24" s="21"/>
-      <c r="X24" s="21"/>
+      <c r="B24" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="17"/>
+      <c r="U24" s="17"/>
+      <c r="V24" s="17"/>
+      <c r="W24" s="17"/>
+      <c r="X24" s="17"/>
     </row>
     <row r="27" customHeight="1" spans="2:24">
-      <c r="M27" s="22"/>
+      <c r="M27" s="11"/>
     </row>
     <row r="28" customHeight="1" spans="2:24">
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="23"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="23"/>
-      <c r="V28" s="23"/>
-      <c r="W28" s="23"/>
-      <c r="X28" s="23"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="22"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+      <c r="M28" s="22"/>
+      <c r="N28" s="22"/>
+      <c r="O28" s="22"/>
+      <c r="P28" s="22"/>
+      <c r="Q28" s="22"/>
+      <c r="R28" s="22"/>
+      <c r="S28" s="22"/>
+      <c r="T28" s="22"/>
+      <c r="U28" s="22"/>
+      <c r="V28" s="22"/>
+      <c r="W28" s="22"/>
+      <c r="X28" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2732,8 +2901,172 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
+  <dimension ref="G10:K18"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18"/>
+  <cols>
+    <col min="7" max="7" width="12.875" customWidth="1"/>
+    <col min="8" max="8" width="15.25" customWidth="1"/>
+    <col min="9" max="9" width="59.625" customWidth="1"/>
+    <col min="10" max="10" width="21.125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="10" spans="7:10">
+      <c r="G10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="11" spans="7:10">
+      <c r="H11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="7:10">
+      <c r="I12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="7:10">
+      <c r="H13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" ht="323" customHeight="1" spans="7:10">
+      <c r="I14" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="7:10">
+      <c r="H15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" ht="409" customHeight="1" spans="7:10">
+      <c r="I16" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="9:11">
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I18:K18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:M19"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18"/>
+  <cols>
+    <col min="9" max="11" width="36.75" customWidth="1"/>
+    <col min="12" max="12" width="49.5" customWidth="1"/>
+    <col min="13" max="13" width="16.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="I13" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="M13" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" ht="54" spans="1:13">
+      <c r="I14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" ht="54" spans="1:13">
+      <c r="I15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="L15" s="3"/>
+      <c r="M15" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="I16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="9:12">
+      <c r="I17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="9:12">
+      <c r="I18" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="9:12">
+      <c r="I19" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="16384" width="9" style="1"/>
   </cols>

</xml_diff>

<commit_message>
new update for API
</commit_message>
<xml_diff>
--- a/doc/OneNode数据格式.xlsx
+++ b/doc/OneNode数据格式.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17895" activeTab="2"/>
+    <workbookView windowWidth="26655" windowHeight="12495" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Message" sheetId="1" r:id="rId1"/>
@@ -344,12 +344,15 @@
   </si>
   <si>
     <t>{
-  "option":  {
+  "options":  {
      "page": 1，
      "page_length": 12,
      "filter": {
            "fetch_state": null/success/failed,
-           "import_state": null/success/failed
+           "import_state": null/success/failed,
+           "from_date": "2023-12-01"/null,
+           "to_date": "2025-12-01"/null,
+           "case_num": "xxxx/null"
       }
   },
   "app_name": "公估报告智数问答",
@@ -406,6 +409,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">ctx: 当前上下文
 name: 数据节点名字
 </t>
@@ -432,6 +442,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">ctx: </t>
     </r>
     <r>
@@ -1290,8 +1307,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
@@ -2921,7 +2938,7 @@
       </c>
     </row>
     <row r="12" spans="7:10">
-      <c r="I12" t="s">
+      <c r="I12" s="6" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2931,7 +2948,7 @@
       </c>
     </row>
     <row r="14" ht="323" customHeight="1" spans="7:10">
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="3" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2941,22 +2958,25 @@
       </c>
     </row>
     <row r="16" ht="409" customHeight="1" spans="7:10">
-      <c r="I16" s="6" t="s">
+      <c r="I16" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="J16" s="6" t="s">
+      <c r="J16" s="3" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="18" spans="9:11">
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I18:K18"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="I12" r:id="rId1" display="https://www.seek-time.com:43031/agents/api/v1/application/run"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>